<commit_message>
AI Restructure, BarRace working
</commit_message>
<xml_diff>
--- a/sjvisualizer/data/Area Dev.xlsx
+++ b/sjvisualizer/data/Area Dev.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9ee5cb27056b4755/Documenten/GitHub/Animation-2/sjvisualizer/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sjoer\Documents\GitHub\sjvisualizer\sjvisualizer\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{50456EFC-884F-4A4F-ACAF-515AC7165218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66B805A8-AE0C-42CD-8058-BC3EA25F999F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4B5DA04-F32E-457A-9AE1-FB9989AC5CD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -194,10 +194,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -464,36 +460,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R176"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7265625" customWidth="1"/>
-    <col min="3" max="3" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.54296875" customWidth="1"/>
-    <col min="6" max="6" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.7265625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.73046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.73046875" customWidth="1"/>
+    <col min="3" max="3" width="9.73046875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.73046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.53125" customWidth="1"/>
+    <col min="6" max="6" width="13.73046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.53125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.73046875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.73046875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.796875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16" bestFit="1" customWidth="1"/>
     <col min="12" max="13" width="16" customWidth="1"/>
-    <col min="14" max="14" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.54296875" customWidth="1"/>
-    <col min="16" max="16" width="16.7265625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="19.26953125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.46484375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.53125" customWidth="1"/>
+    <col min="16" max="16" width="16.73046875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.265625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="19.265625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.46484375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.46484375" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="14" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="5.1796875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="5.19921875" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="8" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.26953125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.796875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.45">
       <c r="B1" t="s">
         <v>35</v>
       </c>
@@ -546,7 +542,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
         <v>42735</v>
       </c>
@@ -602,7 +598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A3" s="1">
         <v>43128</v>
       </c>
@@ -658,7 +654,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A4" s="1">
         <v>43478</v>
       </c>
@@ -714,7 +710,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
         <v>43815</v>
       </c>
@@ -770,7 +766,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
         <v>44001</v>
       </c>
@@ -826,7 +822,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
         <v>44182</v>
       </c>
@@ -882,7 +878,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>44365</v>
       </c>
@@ -938,7 +934,7 @@
         <v>333.33333333333297</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
         <v>44426</v>
       </c>
@@ -994,7 +990,7 @@
         <v>333.33333333333297</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <v>44487</v>
       </c>
@@ -1050,667 +1046,667 @@
         <v>355.55555555555497</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.45">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A49" s="1"/>
       <c r="B49" s="1"/>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A50" s="1"/>
       <c r="B50" s="1"/>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A51" s="1"/>
       <c r="B51" s="1"/>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A52" s="1"/>
       <c r="B52" s="1"/>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A53" s="1"/>
       <c r="B53" s="1"/>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A54" s="1"/>
       <c r="B54" s="1"/>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A55" s="1"/>
       <c r="B55" s="1"/>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A56" s="1"/>
       <c r="B56" s="1"/>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A57" s="1"/>
       <c r="B57" s="1"/>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A58" s="1"/>
       <c r="B58" s="1"/>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A59" s="1"/>
       <c r="B59" s="1"/>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A60" s="1"/>
       <c r="B60" s="1"/>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A61" s="1"/>
       <c r="B61" s="1"/>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A62" s="1"/>
       <c r="B62" s="1"/>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A63" s="1"/>
       <c r="B63" s="1"/>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A64" s="1"/>
       <c r="B64" s="1"/>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A65" s="1"/>
       <c r="B65" s="1"/>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A66" s="1"/>
       <c r="B66" s="1"/>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A67" s="1"/>
       <c r="B67" s="1"/>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A68" s="1"/>
       <c r="B68" s="1"/>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A69" s="1"/>
       <c r="B69" s="1"/>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A70" s="1"/>
       <c r="B70" s="1"/>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A71" s="1"/>
       <c r="B71" s="1"/>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A72" s="1"/>
       <c r="B72" s="1"/>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A73" s="1"/>
       <c r="B73" s="1"/>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A74" s="1"/>
       <c r="B74" s="1"/>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A75" s="1"/>
       <c r="B75" s="1"/>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A76" s="1"/>
       <c r="B76" s="1"/>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A77" s="1"/>
       <c r="B77" s="1"/>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A78" s="1"/>
       <c r="B78" s="1"/>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A79" s="1"/>
       <c r="B79" s="1"/>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A80" s="1"/>
       <c r="B80" s="1"/>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A81" s="1"/>
       <c r="B81" s="1"/>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A82" s="1"/>
       <c r="B82" s="1"/>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A83" s="1"/>
       <c r="B83" s="1"/>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A84" s="1"/>
       <c r="B84" s="1"/>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A85" s="1"/>
       <c r="B85" s="1"/>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A86" s="1"/>
       <c r="B86" s="1"/>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A87" s="1"/>
       <c r="B87" s="1"/>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A88" s="1"/>
       <c r="B88" s="1"/>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A89" s="1"/>
       <c r="B89" s="1"/>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A90" s="1"/>
       <c r="B90" s="1"/>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A91" s="1"/>
       <c r="B91" s="1"/>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A92" s="1"/>
       <c r="B92" s="1"/>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A93" s="1"/>
       <c r="B93" s="1"/>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A94" s="1"/>
       <c r="B94" s="1"/>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A95" s="1"/>
       <c r="B95" s="1"/>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A96" s="1"/>
       <c r="B96" s="1"/>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A97" s="1"/>
       <c r="B97" s="1"/>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A98" s="1"/>
       <c r="B98" s="1"/>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A99" s="1"/>
       <c r="B99" s="1"/>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A100" s="1"/>
       <c r="B100" s="1"/>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A101" s="1"/>
       <c r="B101" s="1"/>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A102" s="1"/>
       <c r="B102" s="1"/>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A103" s="1"/>
       <c r="B103" s="1"/>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A104" s="1"/>
       <c r="B104" s="1"/>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A105" s="1"/>
       <c r="B105" s="1"/>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A106" s="1"/>
       <c r="B106" s="1"/>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A107" s="1"/>
       <c r="B107" s="1"/>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A108" s="1"/>
       <c r="B108" s="1"/>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A109" s="1"/>
       <c r="B109" s="1"/>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A110" s="1"/>
       <c r="B110" s="1"/>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A111" s="1"/>
       <c r="B111" s="1"/>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A112" s="1"/>
       <c r="B112" s="1"/>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A113" s="1"/>
       <c r="B113" s="1"/>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A114" s="1"/>
       <c r="B114" s="1"/>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A115" s="1"/>
       <c r="B115" s="1"/>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A116" s="1"/>
       <c r="B116" s="1"/>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A117" s="1"/>
       <c r="B117" s="1"/>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A118" s="1"/>
       <c r="B118" s="1"/>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A119" s="1"/>
       <c r="B119" s="1"/>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A120" s="1"/>
       <c r="B120" s="1"/>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A121" s="1"/>
       <c r="B121" s="1"/>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A122" s="1"/>
       <c r="B122" s="1"/>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A123" s="1"/>
       <c r="B123" s="1"/>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A124" s="1"/>
       <c r="B124" s="1"/>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A125" s="1"/>
       <c r="B125" s="1"/>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A126" s="1"/>
       <c r="B126" s="1"/>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A127" s="1"/>
       <c r="B127" s="1"/>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A128" s="1"/>
       <c r="B128" s="1"/>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A129" s="1"/>
       <c r="B129" s="1"/>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A130" s="1"/>
       <c r="B130" s="1"/>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A131" s="1"/>
       <c r="B131" s="1"/>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A132" s="1"/>
       <c r="B132" s="1"/>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A133" s="1"/>
       <c r="B133" s="1"/>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A134" s="1"/>
       <c r="B134" s="1"/>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A135" s="1"/>
       <c r="B135" s="1"/>
     </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A136" s="1"/>
       <c r="B136" s="1"/>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A137" s="1"/>
       <c r="B137" s="1"/>
     </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A138" s="1"/>
       <c r="B138" s="1"/>
     </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A139" s="1"/>
       <c r="B139" s="1"/>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A140" s="1"/>
       <c r="B140" s="1"/>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A141" s="1"/>
       <c r="B141" s="1"/>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A142" s="1"/>
       <c r="B142" s="1"/>
     </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A143" s="1"/>
       <c r="B143" s="1"/>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A144" s="1"/>
       <c r="B144" s="1"/>
     </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A145" s="1"/>
       <c r="B145" s="1"/>
     </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A146" s="1"/>
       <c r="B146" s="1"/>
     </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A147" s="1"/>
       <c r="B147" s="1"/>
     </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A148" s="1"/>
       <c r="B148" s="1"/>
     </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A149" s="1"/>
       <c r="B149" s="1"/>
     </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A150" s="1"/>
       <c r="B150" s="1"/>
     </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A151" s="1"/>
       <c r="B151" s="1"/>
     </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A152" s="1"/>
       <c r="B152" s="1"/>
     </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A153" s="1"/>
       <c r="B153" s="1"/>
     </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A154" s="1"/>
       <c r="B154" s="1"/>
     </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A155" s="1"/>
       <c r="B155" s="1"/>
     </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A156" s="1"/>
       <c r="B156" s="1"/>
     </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A157" s="1"/>
       <c r="B157" s="1"/>
     </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A158" s="1"/>
       <c r="B158" s="1"/>
     </row>
-    <row r="159" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A159" s="1"/>
       <c r="B159" s="1"/>
     </row>
-    <row r="160" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A160" s="1"/>
       <c r="B160" s="1"/>
     </row>
-    <row r="161" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A161" s="1"/>
       <c r="B161" s="1"/>
     </row>
-    <row r="162" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A162" s="1"/>
       <c r="B162" s="1"/>
     </row>
-    <row r="163" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A163" s="1"/>
       <c r="B163" s="1"/>
     </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A164" s="1"/>
       <c r="B164" s="1"/>
     </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A165" s="1"/>
       <c r="B165" s="1"/>
     </row>
-    <row r="166" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A166" s="1"/>
       <c r="B166" s="1"/>
     </row>
-    <row r="167" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A167" s="1"/>
       <c r="B167" s="1"/>
     </row>
-    <row r="168" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A168" s="1"/>
       <c r="B168" s="1"/>
     </row>
-    <row r="169" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A169" s="1"/>
       <c r="B169" s="1"/>
     </row>
-    <row r="170" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A170" s="1"/>
       <c r="B170" s="1"/>
     </row>
-    <row r="171" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A171" s="1"/>
       <c r="B171" s="1"/>
     </row>
-    <row r="172" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A172" s="1"/>
       <c r="B172" s="1"/>
     </row>
-    <row r="173" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A173" s="1"/>
       <c r="B173" s="1"/>
     </row>
-    <row r="174" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A174" s="1"/>
       <c r="B174" s="1"/>
     </row>
-    <row r="175" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A175" s="1"/>
       <c r="B175" s="1"/>
     </row>
-    <row r="176" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A176" s="1"/>
       <c r="B176" s="1"/>
     </row>
@@ -1722,9 +1718,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1647956-CA7F-4AFC-917D-E8D31217CB1A}">
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1">
         <v>1</v>
       </c>
@@ -1744,7 +1740,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>2</v>
       </c>
@@ -1761,7 +1757,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>3</v>
       </c>
@@ -1781,7 +1777,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>4</v>
       </c>
@@ -1801,7 +1797,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>5</v>
       </c>
@@ -1818,7 +1814,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>6</v>
       </c>
@@ -1835,7 +1831,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>7</v>
       </c>
@@ -1852,7 +1848,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>8</v>
       </c>
@@ -1869,7 +1865,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>9</v>
       </c>
@@ -1886,7 +1882,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>10</v>
       </c>

</xml_diff>